<commit_message>
ajout du dossier portfolio
</commit_message>
<xml_diff>
--- a/img/E5 - TS SISR 2026.xlsx
+++ b/img/E5 - TS SISR 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20380"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\STAGE\Portfolio\HTML\img\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{219A3E37-7D81-41B9-BB15-D93C82029046}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B41DB87E-B1DD-490A-BCBB-7FF06320F14F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="47">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -143,37 +143,13 @@
     <t>Réalisation en cours de formation</t>
   </si>
   <si>
-    <t>AP 2.1 Godzilla</t>
-  </si>
-  <si>
     <t>X</t>
-  </si>
-  <si>
-    <t>AP 2.2 Strife</t>
-  </si>
-  <si>
-    <t>AP 2.3 FlexOffice</t>
-  </si>
-  <si>
-    <t>AP 2.4 Assiz</t>
-  </si>
-  <si>
-    <t>AP 3.1 Navajo</t>
-  </si>
-  <si>
-    <t>AP 3.2 GPoPu</t>
-  </si>
-  <si>
-    <t>AP 4.1 DMZ</t>
   </si>
   <si>
     <t>Réalisations en milieu professionnel en cours de première année</t>
   </si>
   <si>
     <t>Réalisations en milieu professionnel en cours de seconde année</t>
-  </si>
-  <si>
-    <t>Mise en place d'un ordinateur dans l'autopilot</t>
   </si>
   <si>
     <t>Mettre en place une supervision avec génération d'alertes pertinentes</t>
@@ -183,6 +159,15 @@
   </si>
   <si>
     <t>Déploiement des postes avec automatisation ( Microsoft Intunes ) + Veyon</t>
+  </si>
+  <si>
+    <t>AP 3.2 GPoPu - Mise en place du service DNS et DHCP</t>
+  </si>
+  <si>
+    <t>AP 3.1 Navajo - Mise en place de VLAN ( MUTLAB )</t>
+  </si>
+  <si>
+    <t>AP 2.1 Godzilla - Déploiement avec WAPT</t>
   </si>
 </sst>
 </file>
@@ -253,12 +238,24 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="26">
@@ -614,7 +611,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -642,9 +639,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -706,6 +700,27 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -738,6 +753,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -974,136 +992,136 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
       <c r="G1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="40.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="38"/>
+      <c r="E2" s="38"/>
+      <c r="F2" s="38"/>
+      <c r="G2" s="38"/>
+      <c r="H2" s="38"/>
     </row>
     <row r="3" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="33" t="s">
+      <c r="A3" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="33" t="s">
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
-      <c r="K3" s="34"/>
-      <c r="L3" s="34"/>
-      <c r="M3" s="34"/>
-      <c r="N3" s="34"/>
-      <c r="O3" s="34"/>
-      <c r="P3" s="34"/>
-      <c r="Q3" s="34"/>
-      <c r="R3" s="34"/>
-      <c r="S3" s="34"/>
-      <c r="T3" s="34"/>
-      <c r="U3" s="34"/>
-      <c r="V3" s="34"/>
-      <c r="W3" s="34"/>
-      <c r="X3" s="35"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
+      <c r="K3" s="40"/>
+      <c r="L3" s="40"/>
+      <c r="M3" s="40"/>
+      <c r="N3" s="40"/>
+      <c r="O3" s="40"/>
+      <c r="P3" s="40"/>
+      <c r="Q3" s="40"/>
+      <c r="R3" s="40"/>
+      <c r="S3" s="40"/>
+      <c r="T3" s="40"/>
+      <c r="U3" s="40"/>
+      <c r="V3" s="40"/>
+      <c r="W3" s="40"/>
+      <c r="X3" s="41"/>
     </row>
     <row r="4" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="36" t="s">
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="34"/>
-      <c r="M4" s="34"/>
-      <c r="N4" s="34"/>
-      <c r="O4" s="34"/>
-      <c r="P4" s="34"/>
-      <c r="Q4" s="34"/>
-      <c r="R4" s="34"/>
-      <c r="S4" s="34"/>
-      <c r="T4" s="34"/>
-      <c r="U4" s="34"/>
-      <c r="V4" s="34"/>
-      <c r="W4" s="34"/>
-      <c r="X4" s="34"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
+      <c r="I4" s="40"/>
+      <c r="J4" s="40"/>
+      <c r="K4" s="40"/>
+      <c r="L4" s="40"/>
+      <c r="M4" s="40"/>
+      <c r="N4" s="40"/>
+      <c r="O4" s="40"/>
+      <c r="P4" s="40"/>
+      <c r="Q4" s="40"/>
+      <c r="R4" s="40"/>
+      <c r="S4" s="40"/>
+      <c r="T4" s="40"/>
+      <c r="U4" s="40"/>
+      <c r="V4" s="40"/>
+      <c r="W4" s="40"/>
+      <c r="X4" s="40"/>
     </row>
     <row r="5" spans="1:26" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="49" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="45" t="s">
+      <c r="B5" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="37" t="s">
+      <c r="C5" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="38"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="38"/>
-      <c r="G5" s="38"/>
-      <c r="H5" s="39"/>
-      <c r="I5" s="37" t="s">
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="45"/>
+      <c r="I5" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="38"/>
-      <c r="K5" s="39"/>
-      <c r="L5" s="37" t="s">
+      <c r="J5" s="44"/>
+      <c r="K5" s="45"/>
+      <c r="L5" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="M5" s="38"/>
-      <c r="N5" s="39"/>
-      <c r="O5" s="37" t="s">
+      <c r="M5" s="44"/>
+      <c r="N5" s="45"/>
+      <c r="O5" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="P5" s="38"/>
-      <c r="Q5" s="39"/>
-      <c r="R5" s="37" t="s">
+      <c r="P5" s="44"/>
+      <c r="Q5" s="45"/>
+      <c r="R5" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="S5" s="38"/>
-      <c r="T5" s="39"/>
-      <c r="U5" s="37" t="s">
+      <c r="S5" s="44"/>
+      <c r="T5" s="45"/>
+      <c r="U5" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="V5" s="38"/>
-      <c r="W5" s="38"/>
-      <c r="X5" s="39"/>
+      <c r="V5" s="44"/>
+      <c r="W5" s="44"/>
+      <c r="X5" s="45"/>
     </row>
     <row r="6" spans="1:26" ht="324.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="44"/>
-      <c r="B6" s="46"/>
+      <c r="A6" s="50"/>
+      <c r="B6" s="52"/>
       <c r="C6" s="2" t="s">
         <v>15</v>
       </c>
@@ -1174,906 +1192,876 @@
       <c r="Z6" s="7"/>
     </row>
     <row r="7" spans="1:26" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="40" t="s">
+      <c r="A7" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="41"/>
-      <c r="C7" s="41"/>
-      <c r="D7" s="41"/>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="41"/>
-      <c r="H7" s="41"/>
-      <c r="I7" s="41"/>
-      <c r="J7" s="41"/>
-      <c r="K7" s="41"/>
-      <c r="L7" s="41"/>
-      <c r="M7" s="41"/>
-      <c r="N7" s="41"/>
-      <c r="O7" s="41"/>
-      <c r="P7" s="41"/>
-      <c r="Q7" s="41"/>
-      <c r="R7" s="41"/>
-      <c r="S7" s="41"/>
-      <c r="T7" s="41"/>
-      <c r="U7" s="41"/>
-      <c r="V7" s="41"/>
-      <c r="W7" s="41"/>
-      <c r="X7" s="42"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="47"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="47"/>
+      <c r="K7" s="47"/>
+      <c r="L7" s="47"/>
+      <c r="M7" s="47"/>
+      <c r="N7" s="47"/>
+      <c r="O7" s="47"/>
+      <c r="P7" s="47"/>
+      <c r="Q7" s="47"/>
+      <c r="R7" s="47"/>
+      <c r="S7" s="47"/>
+      <c r="T7" s="47"/>
+      <c r="U7" s="47"/>
+      <c r="V7" s="47"/>
+      <c r="W7" s="47"/>
+      <c r="X7" s="48"/>
       <c r="Y7" s="7"/>
       <c r="Z7" s="7"/>
     </row>
     <row r="8" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="9"/>
+      <c r="C8" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="10" t="s">
-        <v>39</v>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="13"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="12"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="12"/>
+      <c r="P8" s="13"/>
+      <c r="Q8" s="14"/>
+      <c r="R8" s="12"/>
+      <c r="S8" s="31" t="s">
+        <v>38</v>
       </c>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="13"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="13"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="15"/>
-      <c r="O8" s="13"/>
-      <c r="P8" s="14"/>
-      <c r="Q8" s="15"/>
-      <c r="R8" s="13"/>
-      <c r="S8" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="T8" s="15"/>
-      <c r="U8" s="13"/>
-      <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
-      <c r="X8" s="15"/>
+      <c r="T8" s="14"/>
+      <c r="U8" s="12"/>
+      <c r="V8" s="13"/>
+      <c r="W8" s="13"/>
+      <c r="X8" s="14"/>
       <c r="Y8" s="7"/>
       <c r="Z8" s="7"/>
     </row>
     <row r="9" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B9" s="9"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="20"/>
-      <c r="K9" s="21"/>
-      <c r="L9" s="19"/>
-      <c r="M9" s="20"/>
-      <c r="N9" s="21"/>
-      <c r="O9" s="19"/>
-      <c r="P9" s="20"/>
-      <c r="Q9" s="21"/>
-      <c r="R9" s="19" t="s">
-        <v>39</v>
+      <c r="C9" s="15"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="G9" s="16"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="18"/>
+      <c r="J9" s="32" t="s">
+        <v>38</v>
       </c>
-      <c r="S9" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="T9" s="21"/>
-      <c r="U9" s="19"/>
-      <c r="V9" s="20"/>
-      <c r="W9" s="20"/>
-      <c r="X9" s="21"/>
+      <c r="K9" s="20"/>
+      <c r="L9" s="18"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="20"/>
+      <c r="O9" s="18"/>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="20"/>
+      <c r="R9" s="18"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="20"/>
+      <c r="U9" s="18"/>
+      <c r="V9" s="19"/>
+      <c r="W9" s="19"/>
+      <c r="X9" s="20"/>
       <c r="Y9" s="7"/>
       <c r="Z9" s="7"/>
     </row>
     <row r="10" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B10" s="9"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17" t="s">
-        <v>39</v>
+      <c r="C10" s="15"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="32" t="s">
+        <v>38</v>
       </c>
-      <c r="H10" s="18"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="20"/>
-      <c r="N10" s="21"/>
-      <c r="O10" s="19"/>
-      <c r="P10" s="20"/>
-      <c r="Q10" s="21"/>
-      <c r="R10" s="19"/>
-      <c r="S10" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="T10" s="21"/>
-      <c r="U10" s="19"/>
-      <c r="V10" s="20"/>
-      <c r="W10" s="20"/>
-      <c r="X10" s="21"/>
+      <c r="K10" s="20"/>
+      <c r="L10" s="18"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="20"/>
+      <c r="O10" s="18"/>
+      <c r="P10" s="19"/>
+      <c r="Q10" s="20"/>
+      <c r="R10" s="18"/>
+      <c r="S10" s="19"/>
+      <c r="T10" s="20"/>
+      <c r="U10" s="18"/>
+      <c r="V10" s="19"/>
+      <c r="W10" s="19"/>
+      <c r="X10" s="20"/>
       <c r="Y10" s="7"/>
       <c r="Z10" s="7"/>
     </row>
     <row r="11" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="8" t="s">
-        <v>42</v>
-      </c>
+      <c r="A11" s="8"/>
       <c r="B11" s="9"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="20"/>
-      <c r="K11" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="L11" s="19"/>
-      <c r="M11" s="20"/>
-      <c r="N11" s="21"/>
-      <c r="O11" s="19"/>
-      <c r="P11" s="20"/>
-      <c r="Q11" s="21"/>
-      <c r="R11" s="19"/>
-      <c r="S11" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="T11" s="21"/>
-      <c r="U11" s="19"/>
-      <c r="V11" s="20"/>
-      <c r="W11" s="20"/>
-      <c r="X11" s="21"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="54"/>
+      <c r="G11" s="54"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="54"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="18"/>
+      <c r="M11" s="19"/>
+      <c r="N11" s="20"/>
+      <c r="O11" s="18"/>
+      <c r="P11" s="19"/>
+      <c r="Q11" s="20"/>
+      <c r="R11" s="18"/>
+      <c r="S11" s="54"/>
+      <c r="T11" s="20"/>
+      <c r="U11" s="18"/>
+      <c r="V11" s="19"/>
+      <c r="W11" s="19"/>
+      <c r="X11" s="20"/>
       <c r="Y11" s="7"/>
       <c r="Z11" s="7"/>
     </row>
     <row r="12" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="8" t="s">
-        <v>43</v>
-      </c>
+      <c r="A12" s="8"/>
       <c r="B12" s="9"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="19"/>
-      <c r="J12" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="K12" s="21"/>
-      <c r="L12" s="19"/>
-      <c r="M12" s="20"/>
-      <c r="N12" s="21"/>
-      <c r="O12" s="19"/>
-      <c r="P12" s="20"/>
-      <c r="Q12" s="21"/>
-      <c r="R12" s="19"/>
-      <c r="S12" s="20"/>
-      <c r="T12" s="21"/>
-      <c r="U12" s="19"/>
-      <c r="V12" s="20"/>
-      <c r="W12" s="20"/>
-      <c r="X12" s="21"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="19"/>
+      <c r="K12" s="20"/>
+      <c r="L12" s="18"/>
+      <c r="M12" s="19"/>
+      <c r="N12" s="20"/>
+      <c r="O12" s="18"/>
+      <c r="P12" s="19"/>
+      <c r="Q12" s="20"/>
+      <c r="R12" s="18"/>
+      <c r="S12" s="19"/>
+      <c r="T12" s="20"/>
+      <c r="U12" s="18"/>
+      <c r="V12" s="19"/>
+      <c r="W12" s="19"/>
+      <c r="X12" s="20"/>
       <c r="Y12" s="7"/>
       <c r="Z12" s="7"/>
     </row>
     <row r="13" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="8" t="s">
-        <v>44</v>
-      </c>
+      <c r="A13" s="8"/>
       <c r="B13" s="9"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="19"/>
-      <c r="J13" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="K13" s="21"/>
-      <c r="L13" s="19"/>
-      <c r="M13" s="20"/>
-      <c r="N13" s="21"/>
-      <c r="O13" s="19"/>
-      <c r="P13" s="20"/>
-      <c r="Q13" s="21"/>
-      <c r="R13" s="19"/>
-      <c r="S13" s="20"/>
-      <c r="T13" s="21"/>
-      <c r="U13" s="19"/>
-      <c r="V13" s="20"/>
-      <c r="W13" s="20"/>
-      <c r="X13" s="21"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="20"/>
+      <c r="L13" s="18"/>
+      <c r="M13" s="19"/>
+      <c r="N13" s="20"/>
+      <c r="O13" s="18"/>
+      <c r="P13" s="19"/>
+      <c r="Q13" s="20"/>
+      <c r="R13" s="18"/>
+      <c r="S13" s="19"/>
+      <c r="T13" s="20"/>
+      <c r="U13" s="18"/>
+      <c r="V13" s="19"/>
+      <c r="W13" s="19"/>
+      <c r="X13" s="20"/>
       <c r="Y13" s="7"/>
       <c r="Z13" s="7"/>
     </row>
     <row r="14" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="8" t="s">
-        <v>45</v>
-      </c>
+      <c r="A14" s="8"/>
       <c r="B14" s="9"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="G14" s="17" t="s">
-        <v>39</v>
-      </c>
-      <c r="H14" s="18"/>
-      <c r="I14" s="19"/>
-      <c r="J14" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="K14" s="21"/>
-      <c r="L14" s="19"/>
-      <c r="M14" s="20"/>
-      <c r="N14" s="21"/>
-      <c r="O14" s="19"/>
-      <c r="P14" s="20"/>
-      <c r="Q14" s="21"/>
-      <c r="R14" s="19"/>
-      <c r="S14" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="T14" s="21"/>
-      <c r="U14" s="19"/>
-      <c r="V14" s="20"/>
-      <c r="W14" s="20"/>
-      <c r="X14" s="21"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="20"/>
+      <c r="L14" s="18"/>
+      <c r="M14" s="19"/>
+      <c r="N14" s="20"/>
+      <c r="O14" s="18"/>
+      <c r="P14" s="19"/>
+      <c r="Q14" s="20"/>
+      <c r="R14" s="18"/>
+      <c r="S14" s="19"/>
+      <c r="T14" s="20"/>
+      <c r="U14" s="18"/>
+      <c r="V14" s="19"/>
+      <c r="W14" s="19"/>
+      <c r="X14" s="20"/>
       <c r="Y14" s="7"/>
       <c r="Z14" s="7"/>
     </row>
     <row r="15" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8"/>
       <c r="B15" s="9"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="19"/>
-      <c r="J15" s="20"/>
-      <c r="K15" s="21"/>
-      <c r="L15" s="19"/>
-      <c r="M15" s="20"/>
-      <c r="N15" s="21"/>
-      <c r="O15" s="19"/>
-      <c r="P15" s="20"/>
-      <c r="Q15" s="21"/>
-      <c r="R15" s="19"/>
-      <c r="S15" s="20"/>
-      <c r="T15" s="21"/>
-      <c r="U15" s="19"/>
-      <c r="V15" s="20"/>
-      <c r="W15" s="20"/>
-      <c r="X15" s="21"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="19"/>
+      <c r="K15" s="20"/>
+      <c r="L15" s="18"/>
+      <c r="M15" s="19"/>
+      <c r="N15" s="20"/>
+      <c r="O15" s="18"/>
+      <c r="P15" s="19"/>
+      <c r="Q15" s="20"/>
+      <c r="R15" s="18"/>
+      <c r="S15" s="19"/>
+      <c r="T15" s="20"/>
+      <c r="U15" s="18"/>
+      <c r="V15" s="19"/>
+      <c r="W15" s="19"/>
+      <c r="X15" s="20"/>
       <c r="Y15" s="7"/>
       <c r="Z15" s="7"/>
     </row>
     <row r="16" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="8"/>
       <c r="B16" s="9"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="20"/>
-      <c r="K16" s="21"/>
-      <c r="L16" s="19"/>
-      <c r="M16" s="20"/>
-      <c r="N16" s="21"/>
-      <c r="O16" s="19"/>
-      <c r="P16" s="20"/>
-      <c r="Q16" s="21"/>
-      <c r="R16" s="19"/>
-      <c r="S16" s="20"/>
-      <c r="T16" s="21"/>
-      <c r="U16" s="19"/>
-      <c r="V16" s="20"/>
-      <c r="W16" s="20"/>
-      <c r="X16" s="21"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="18"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="20"/>
+      <c r="L16" s="18"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="20"/>
+      <c r="O16" s="18"/>
+      <c r="P16" s="19"/>
+      <c r="Q16" s="20"/>
+      <c r="R16" s="18"/>
+      <c r="S16" s="19"/>
+      <c r="T16" s="20"/>
+      <c r="U16" s="18"/>
+      <c r="V16" s="19"/>
+      <c r="W16" s="19"/>
+      <c r="X16" s="20"/>
       <c r="Y16" s="7"/>
       <c r="Z16" s="7"/>
     </row>
     <row r="17" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="8"/>
       <c r="B17" s="9"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="20"/>
-      <c r="K17" s="21"/>
-      <c r="L17" s="19"/>
-      <c r="M17" s="20"/>
-      <c r="N17" s="21"/>
-      <c r="O17" s="19"/>
-      <c r="P17" s="20"/>
-      <c r="Q17" s="21"/>
-      <c r="R17" s="19"/>
-      <c r="S17" s="20"/>
-      <c r="T17" s="21"/>
-      <c r="U17" s="19"/>
-      <c r="V17" s="20"/>
-      <c r="W17" s="20"/>
-      <c r="X17" s="21"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="19"/>
+      <c r="K17" s="20"/>
+      <c r="L17" s="18"/>
+      <c r="M17" s="19"/>
+      <c r="N17" s="20"/>
+      <c r="O17" s="18"/>
+      <c r="P17" s="19"/>
+      <c r="Q17" s="20"/>
+      <c r="R17" s="18"/>
+      <c r="S17" s="19"/>
+      <c r="T17" s="20"/>
+      <c r="U17" s="18"/>
+      <c r="V17" s="19"/>
+      <c r="W17" s="19"/>
+      <c r="X17" s="20"/>
       <c r="Y17" s="7"/>
       <c r="Z17" s="7"/>
     </row>
     <row r="18" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="47" t="s">
-        <v>46</v>
+      <c r="A18" s="53" t="s">
+        <v>39</v>
       </c>
-      <c r="B18" s="41"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="41"/>
-      <c r="F18" s="41"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="20"/>
-      <c r="K18" s="21"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="20"/>
-      <c r="N18" s="21"/>
-      <c r="O18" s="19"/>
-      <c r="P18" s="20"/>
-      <c r="Q18" s="21"/>
-      <c r="R18" s="19"/>
-      <c r="S18" s="20"/>
-      <c r="T18" s="21"/>
-      <c r="U18" s="19"/>
-      <c r="V18" s="20"/>
-      <c r="W18" s="20"/>
-      <c r="X18" s="21"/>
+      <c r="B18" s="47"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="47"/>
+      <c r="F18" s="47"/>
+      <c r="G18" s="47"/>
+      <c r="H18" s="48"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="20"/>
+      <c r="L18" s="18"/>
+      <c r="M18" s="19"/>
+      <c r="N18" s="20"/>
+      <c r="O18" s="18"/>
+      <c r="P18" s="19"/>
+      <c r="Q18" s="20"/>
+      <c r="R18" s="18"/>
+      <c r="S18" s="19"/>
+      <c r="T18" s="20"/>
+      <c r="U18" s="18"/>
+      <c r="V18" s="19"/>
+      <c r="W18" s="19"/>
+      <c r="X18" s="20"/>
       <c r="Y18" s="7"/>
       <c r="Z18" s="7"/>
     </row>
     <row r="19" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B19" s="9"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17" t="s">
-        <v>39</v>
+      <c r="C19" s="15"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="33" t="s">
+        <v>38</v>
       </c>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="18" t="s">
-        <v>39</v>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="34" t="s">
+        <v>38</v>
       </c>
-      <c r="I19" s="19"/>
-      <c r="J19" s="20"/>
-      <c r="K19" s="21"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="20"/>
-      <c r="N19" s="21"/>
-      <c r="O19" s="19"/>
-      <c r="P19" s="20"/>
-      <c r="Q19" s="21"/>
-      <c r="R19" s="19" t="s">
-        <v>39</v>
+      <c r="I19" s="18"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="20"/>
+      <c r="L19" s="18"/>
+      <c r="M19" s="19"/>
+      <c r="N19" s="20"/>
+      <c r="O19" s="18"/>
+      <c r="P19" s="19"/>
+      <c r="Q19" s="20"/>
+      <c r="R19" s="35" t="s">
+        <v>38</v>
       </c>
-      <c r="S19" s="20" t="s">
-        <v>39</v>
+      <c r="S19" s="32" t="s">
+        <v>38</v>
       </c>
-      <c r="T19" s="21"/>
-      <c r="U19" s="19"/>
-      <c r="V19" s="20"/>
-      <c r="W19" s="20"/>
-      <c r="X19" s="21"/>
+      <c r="T19" s="20"/>
+      <c r="U19" s="18"/>
+      <c r="V19" s="19"/>
+      <c r="W19" s="19"/>
+      <c r="X19" s="20"/>
       <c r="Y19" s="7"/>
       <c r="Z19" s="7"/>
     </row>
     <row r="20" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B20" s="9"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17" t="s">
-        <v>39</v>
+      <c r="C20" s="15"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="33" t="s">
+        <v>38</v>
       </c>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="18" t="s">
-        <v>39</v>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="34" t="s">
+        <v>38</v>
       </c>
-      <c r="I20" s="19"/>
-      <c r="J20" s="20" t="s">
-        <v>39</v>
+      <c r="I20" s="18"/>
+      <c r="J20" s="32" t="s">
+        <v>38</v>
       </c>
-      <c r="K20" s="21"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="20"/>
-      <c r="N20" s="21"/>
-      <c r="O20" s="19"/>
-      <c r="P20" s="20"/>
-      <c r="Q20" s="21"/>
-      <c r="R20" s="19"/>
-      <c r="S20" s="20"/>
-      <c r="T20" s="21"/>
-      <c r="U20" s="19"/>
-      <c r="V20" s="20"/>
-      <c r="W20" s="20"/>
-      <c r="X20" s="21"/>
+      <c r="K20" s="20"/>
+      <c r="L20" s="18"/>
+      <c r="M20" s="19"/>
+      <c r="N20" s="20"/>
+      <c r="O20" s="18"/>
+      <c r="P20" s="19"/>
+      <c r="Q20" s="20"/>
+      <c r="R20" s="18"/>
+      <c r="S20" s="19"/>
+      <c r="T20" s="20"/>
+      <c r="U20" s="18"/>
+      <c r="V20" s="19"/>
+      <c r="W20" s="19"/>
+      <c r="X20" s="20"/>
       <c r="Y20" s="7"/>
       <c r="Z20" s="7"/>
     </row>
     <row r="21" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="8"/>
       <c r="B21" s="9"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="19"/>
-      <c r="J21" s="20"/>
-      <c r="K21" s="21"/>
-      <c r="L21" s="19"/>
-      <c r="M21" s="20"/>
-      <c r="N21" s="21"/>
-      <c r="O21" s="19"/>
-      <c r="P21" s="20"/>
-      <c r="Q21" s="21"/>
-      <c r="R21" s="19"/>
-      <c r="S21" s="20"/>
-      <c r="T21" s="21"/>
-      <c r="U21" s="19"/>
-      <c r="V21" s="20"/>
-      <c r="W21" s="20"/>
-      <c r="X21" s="21"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="18"/>
+      <c r="J21" s="19"/>
+      <c r="K21" s="20"/>
+      <c r="L21" s="18"/>
+      <c r="M21" s="19"/>
+      <c r="N21" s="20"/>
+      <c r="O21" s="18"/>
+      <c r="P21" s="19"/>
+      <c r="Q21" s="20"/>
+      <c r="R21" s="18"/>
+      <c r="S21" s="19"/>
+      <c r="T21" s="20"/>
+      <c r="U21" s="18"/>
+      <c r="V21" s="19"/>
+      <c r="W21" s="19"/>
+      <c r="X21" s="20"/>
       <c r="Y21" s="7"/>
       <c r="Z21" s="7"/>
     </row>
     <row r="22" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="8"/>
       <c r="B22" s="9"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="18"/>
-      <c r="I22" s="19"/>
-      <c r="J22" s="20"/>
-      <c r="K22" s="21"/>
-      <c r="L22" s="19"/>
-      <c r="M22" s="20"/>
-      <c r="N22" s="21"/>
-      <c r="O22" s="19"/>
-      <c r="P22" s="20"/>
-      <c r="Q22" s="21"/>
-      <c r="R22" s="19"/>
-      <c r="S22" s="20"/>
-      <c r="T22" s="21"/>
-      <c r="U22" s="19"/>
-      <c r="V22" s="20"/>
-      <c r="W22" s="20"/>
-      <c r="X22" s="21"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="19"/>
+      <c r="K22" s="20"/>
+      <c r="L22" s="18"/>
+      <c r="M22" s="19"/>
+      <c r="N22" s="20"/>
+      <c r="O22" s="18"/>
+      <c r="P22" s="19"/>
+      <c r="Q22" s="20"/>
+      <c r="R22" s="18"/>
+      <c r="S22" s="19"/>
+      <c r="T22" s="20"/>
+      <c r="U22" s="18"/>
+      <c r="V22" s="19"/>
+      <c r="W22" s="19"/>
+      <c r="X22" s="20"/>
       <c r="Y22" s="7"/>
       <c r="Z22" s="7"/>
     </row>
     <row r="23" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="8"/>
       <c r="B23" s="9"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="19"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="21"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="20"/>
-      <c r="N23" s="21"/>
-      <c r="O23" s="19"/>
-      <c r="P23" s="20"/>
-      <c r="Q23" s="21"/>
-      <c r="R23" s="19"/>
-      <c r="S23" s="20"/>
-      <c r="T23" s="21"/>
-      <c r="U23" s="19"/>
-      <c r="V23" s="20"/>
-      <c r="W23" s="20"/>
-      <c r="X23" s="21"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="16"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="18"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="20"/>
+      <c r="L23" s="18"/>
+      <c r="M23" s="19"/>
+      <c r="N23" s="20"/>
+      <c r="O23" s="18"/>
+      <c r="P23" s="19"/>
+      <c r="Q23" s="20"/>
+      <c r="R23" s="18"/>
+      <c r="S23" s="19"/>
+      <c r="T23" s="20"/>
+      <c r="U23" s="18"/>
+      <c r="V23" s="19"/>
+      <c r="W23" s="19"/>
+      <c r="X23" s="20"/>
       <c r="Y23" s="7"/>
       <c r="Z23" s="7"/>
     </row>
     <row r="24" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="8"/>
       <c r="B24" s="9"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="19"/>
-      <c r="J24" s="20"/>
-      <c r="K24" s="21"/>
-      <c r="L24" s="19"/>
-      <c r="M24" s="20"/>
-      <c r="N24" s="21"/>
-      <c r="O24" s="19"/>
-      <c r="P24" s="20"/>
-      <c r="Q24" s="21"/>
-      <c r="R24" s="19"/>
-      <c r="S24" s="20"/>
-      <c r="T24" s="21"/>
-      <c r="U24" s="19"/>
-      <c r="V24" s="20"/>
-      <c r="W24" s="20"/>
-      <c r="X24" s="21"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="18"/>
+      <c r="J24" s="19"/>
+      <c r="K24" s="20"/>
+      <c r="L24" s="18"/>
+      <c r="M24" s="19"/>
+      <c r="N24" s="20"/>
+      <c r="O24" s="18"/>
+      <c r="P24" s="19"/>
+      <c r="Q24" s="20"/>
+      <c r="R24" s="18"/>
+      <c r="S24" s="19"/>
+      <c r="T24" s="20"/>
+      <c r="U24" s="18"/>
+      <c r="V24" s="19"/>
+      <c r="W24" s="19"/>
+      <c r="X24" s="20"/>
       <c r="Y24" s="7"/>
       <c r="Z24" s="7"/>
     </row>
     <row r="25" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="8"/>
       <c r="B25" s="9"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="19"/>
-      <c r="J25" s="20"/>
-      <c r="K25" s="21"/>
-      <c r="L25" s="19"/>
-      <c r="M25" s="20"/>
-      <c r="N25" s="21"/>
-      <c r="O25" s="19"/>
-      <c r="P25" s="20"/>
-      <c r="Q25" s="21"/>
-      <c r="R25" s="19"/>
-      <c r="S25" s="20"/>
-      <c r="T25" s="21"/>
-      <c r="U25" s="19"/>
-      <c r="V25" s="20"/>
-      <c r="W25" s="20"/>
-      <c r="X25" s="21"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="18"/>
+      <c r="J25" s="19"/>
+      <c r="K25" s="20"/>
+      <c r="L25" s="18"/>
+      <c r="M25" s="19"/>
+      <c r="N25" s="20"/>
+      <c r="O25" s="18"/>
+      <c r="P25" s="19"/>
+      <c r="Q25" s="20"/>
+      <c r="R25" s="18"/>
+      <c r="S25" s="19"/>
+      <c r="T25" s="20"/>
+      <c r="U25" s="18"/>
+      <c r="V25" s="19"/>
+      <c r="W25" s="19"/>
+      <c r="X25" s="20"/>
       <c r="Y25" s="7"/>
       <c r="Z25" s="7"/>
     </row>
     <row r="26" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="8"/>
       <c r="B26" s="9"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="18"/>
-      <c r="I26" s="19"/>
-      <c r="J26" s="20"/>
-      <c r="K26" s="21"/>
-      <c r="L26" s="19"/>
-      <c r="M26" s="20"/>
-      <c r="N26" s="21"/>
-      <c r="O26" s="19"/>
-      <c r="P26" s="20"/>
-      <c r="Q26" s="21"/>
-      <c r="R26" s="19"/>
-      <c r="S26" s="20"/>
-      <c r="T26" s="21"/>
-      <c r="U26" s="19"/>
-      <c r="V26" s="20"/>
-      <c r="W26" s="20"/>
-      <c r="X26" s="21"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="18"/>
+      <c r="J26" s="19"/>
+      <c r="K26" s="20"/>
+      <c r="L26" s="18"/>
+      <c r="M26" s="19"/>
+      <c r="N26" s="20"/>
+      <c r="O26" s="18"/>
+      <c r="P26" s="19"/>
+      <c r="Q26" s="20"/>
+      <c r="R26" s="18"/>
+      <c r="S26" s="19"/>
+      <c r="T26" s="20"/>
+      <c r="U26" s="18"/>
+      <c r="V26" s="19"/>
+      <c r="W26" s="19"/>
+      <c r="X26" s="20"/>
       <c r="Y26" s="7"/>
       <c r="Z26" s="7"/>
     </row>
     <row r="27" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="47" t="s">
-        <v>47</v>
+      <c r="A27" s="53" t="s">
+        <v>40</v>
       </c>
-      <c r="B27" s="41"/>
-      <c r="C27" s="41"/>
-      <c r="D27" s="41"/>
-      <c r="E27" s="41"/>
-      <c r="F27" s="41"/>
-      <c r="G27" s="41"/>
-      <c r="H27" s="42"/>
-      <c r="I27" s="19"/>
-      <c r="J27" s="20"/>
-      <c r="K27" s="21"/>
-      <c r="L27" s="19"/>
-      <c r="M27" s="20"/>
-      <c r="N27" s="21"/>
-      <c r="O27" s="19"/>
-      <c r="P27" s="20"/>
-      <c r="Q27" s="21"/>
-      <c r="R27" s="19"/>
-      <c r="S27" s="20"/>
-      <c r="T27" s="21"/>
-      <c r="U27" s="19"/>
-      <c r="V27" s="20"/>
-      <c r="W27" s="20"/>
-      <c r="X27" s="21"/>
+      <c r="B27" s="47"/>
+      <c r="C27" s="47"/>
+      <c r="D27" s="47"/>
+      <c r="E27" s="47"/>
+      <c r="F27" s="47"/>
+      <c r="G27" s="47"/>
+      <c r="H27" s="48"/>
+      <c r="I27" s="18"/>
+      <c r="J27" s="19"/>
+      <c r="K27" s="20"/>
+      <c r="L27" s="18"/>
+      <c r="M27" s="19"/>
+      <c r="N27" s="20"/>
+      <c r="O27" s="18"/>
+      <c r="P27" s="19"/>
+      <c r="Q27" s="20"/>
+      <c r="R27" s="18"/>
+      <c r="S27" s="19"/>
+      <c r="T27" s="20"/>
+      <c r="U27" s="18"/>
+      <c r="V27" s="19"/>
+      <c r="W27" s="19"/>
+      <c r="X27" s="20"/>
       <c r="Y27" s="7"/>
       <c r="Z27" s="7"/>
     </row>
     <row r="28" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="8" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B28" s="9"/>
-      <c r="C28" s="16" t="s">
-        <v>39</v>
+      <c r="C28" s="36" t="s">
+        <v>38</v>
       </c>
-      <c r="D28" s="17" t="s">
-        <v>39</v>
+      <c r="D28" s="33" t="s">
+        <v>38</v>
       </c>
-      <c r="E28" s="17" t="s">
-        <v>39</v>
+      <c r="E28" s="33" t="s">
+        <v>38</v>
       </c>
-      <c r="F28" s="17"/>
-      <c r="G28" s="17" t="s">
-        <v>39</v>
+      <c r="F28" s="16"/>
+      <c r="G28" s="33" t="s">
+        <v>38</v>
       </c>
-      <c r="H28" s="18"/>
-      <c r="I28" s="19"/>
-      <c r="J28" s="20"/>
-      <c r="K28" s="21"/>
-      <c r="L28" s="19"/>
-      <c r="M28" s="20"/>
-      <c r="N28" s="21"/>
-      <c r="O28" s="19"/>
-      <c r="P28" s="20"/>
-      <c r="Q28" s="21"/>
-      <c r="R28" s="19"/>
-      <c r="S28" s="20" t="s">
-        <v>39</v>
+      <c r="H28" s="17"/>
+      <c r="I28" s="18"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="20"/>
+      <c r="L28" s="18"/>
+      <c r="M28" s="19"/>
+      <c r="N28" s="20"/>
+      <c r="O28" s="18"/>
+      <c r="P28" s="19"/>
+      <c r="Q28" s="20"/>
+      <c r="R28" s="18"/>
+      <c r="S28" s="32" t="s">
+        <v>38</v>
       </c>
-      <c r="T28" s="21"/>
-      <c r="U28" s="19"/>
-      <c r="V28" s="20"/>
-      <c r="W28" s="20"/>
-      <c r="X28" s="21"/>
+      <c r="T28" s="20"/>
+      <c r="U28" s="18"/>
+      <c r="V28" s="19"/>
+      <c r="W28" s="19"/>
+      <c r="X28" s="20"/>
       <c r="Y28" s="7"/>
       <c r="Z28" s="7"/>
     </row>
     <row r="29" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="8" t="s">
-        <v>48</v>
-      </c>
+      <c r="A29" s="8"/>
       <c r="B29" s="9"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="18"/>
-      <c r="I29" s="19"/>
-      <c r="J29" s="20"/>
-      <c r="K29" s="21"/>
-      <c r="L29" s="19"/>
-      <c r="M29" s="20"/>
-      <c r="N29" s="21"/>
-      <c r="O29" s="19"/>
-      <c r="P29" s="20"/>
-      <c r="Q29" s="21"/>
-      <c r="R29" s="19"/>
-      <c r="S29" s="20"/>
-      <c r="T29" s="21"/>
-      <c r="U29" s="19"/>
-      <c r="V29" s="20"/>
-      <c r="W29" s="20"/>
-      <c r="X29" s="21"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="18"/>
+      <c r="J29" s="19"/>
+      <c r="K29" s="20"/>
+      <c r="L29" s="18"/>
+      <c r="M29" s="19"/>
+      <c r="N29" s="20"/>
+      <c r="O29" s="18"/>
+      <c r="P29" s="19"/>
+      <c r="Q29" s="20"/>
+      <c r="R29" s="18"/>
+      <c r="S29" s="19"/>
+      <c r="T29" s="20"/>
+      <c r="U29" s="18"/>
+      <c r="V29" s="19"/>
+      <c r="W29" s="19"/>
+      <c r="X29" s="20"/>
       <c r="Y29" s="7"/>
       <c r="Z29" s="7"/>
     </row>
     <row r="30" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="8"/>
       <c r="B30" s="9"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="17"/>
-      <c r="H30" s="18"/>
-      <c r="I30" s="19"/>
-      <c r="J30" s="20"/>
-      <c r="K30" s="21"/>
-      <c r="L30" s="19"/>
-      <c r="M30" s="20"/>
-      <c r="N30" s="21"/>
-      <c r="O30" s="19"/>
-      <c r="P30" s="20"/>
-      <c r="Q30" s="21"/>
-      <c r="R30" s="19"/>
-      <c r="S30" s="20"/>
-      <c r="T30" s="21"/>
-      <c r="U30" s="19"/>
-      <c r="V30" s="20"/>
-      <c r="W30" s="20"/>
-      <c r="X30" s="21"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="19"/>
+      <c r="K30" s="20"/>
+      <c r="L30" s="18"/>
+      <c r="M30" s="19"/>
+      <c r="N30" s="20"/>
+      <c r="O30" s="18"/>
+      <c r="P30" s="19"/>
+      <c r="Q30" s="20"/>
+      <c r="R30" s="18"/>
+      <c r="S30" s="19"/>
+      <c r="T30" s="20"/>
+      <c r="U30" s="18"/>
+      <c r="V30" s="19"/>
+      <c r="W30" s="19"/>
+      <c r="X30" s="20"/>
       <c r="Y30" s="7"/>
       <c r="Z30" s="7"/>
     </row>
     <row r="31" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="8"/>
       <c r="B31" s="9"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="18"/>
-      <c r="I31" s="19"/>
-      <c r="J31" s="20"/>
-      <c r="K31" s="21"/>
-      <c r="L31" s="19"/>
-      <c r="M31" s="20"/>
-      <c r="N31" s="21"/>
-      <c r="O31" s="19"/>
-      <c r="P31" s="20"/>
-      <c r="Q31" s="21"/>
-      <c r="R31" s="19"/>
-      <c r="S31" s="20"/>
-      <c r="T31" s="21"/>
-      <c r="U31" s="19"/>
-      <c r="V31" s="20"/>
-      <c r="W31" s="20"/>
-      <c r="X31" s="21"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="17"/>
+      <c r="I31" s="18"/>
+      <c r="J31" s="19"/>
+      <c r="K31" s="20"/>
+      <c r="L31" s="18"/>
+      <c r="M31" s="19"/>
+      <c r="N31" s="20"/>
+      <c r="O31" s="18"/>
+      <c r="P31" s="19"/>
+      <c r="Q31" s="20"/>
+      <c r="R31" s="18"/>
+      <c r="S31" s="19"/>
+      <c r="T31" s="20"/>
+      <c r="U31" s="18"/>
+      <c r="V31" s="19"/>
+      <c r="W31" s="19"/>
+      <c r="X31" s="20"/>
       <c r="Y31" s="7"/>
       <c r="Z31" s="7"/>
     </row>
     <row r="32" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="8"/>
       <c r="B32" s="9"/>
-      <c r="C32" s="16"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
-      <c r="G32" s="17"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="19"/>
-      <c r="J32" s="20"/>
-      <c r="K32" s="21"/>
-      <c r="L32" s="19"/>
-      <c r="M32" s="20"/>
-      <c r="N32" s="21"/>
-      <c r="O32" s="19"/>
-      <c r="P32" s="20"/>
-      <c r="Q32" s="21"/>
-      <c r="R32" s="19"/>
-      <c r="S32" s="20"/>
-      <c r="T32" s="21"/>
-      <c r="U32" s="19"/>
-      <c r="V32" s="20"/>
-      <c r="W32" s="20"/>
-      <c r="X32" s="21"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="18"/>
+      <c r="J32" s="19"/>
+      <c r="K32" s="20"/>
+      <c r="L32" s="18"/>
+      <c r="M32" s="19"/>
+      <c r="N32" s="20"/>
+      <c r="O32" s="18"/>
+      <c r="P32" s="19"/>
+      <c r="Q32" s="20"/>
+      <c r="R32" s="18"/>
+      <c r="S32" s="19"/>
+      <c r="T32" s="20"/>
+      <c r="U32" s="18"/>
+      <c r="V32" s="19"/>
+      <c r="W32" s="19"/>
+      <c r="X32" s="20"/>
       <c r="Y32" s="7"/>
       <c r="Z32" s="7"/>
     </row>
     <row r="33" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="8"/>
       <c r="B33" s="9"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="18"/>
-      <c r="I33" s="19"/>
-      <c r="J33" s="20"/>
-      <c r="K33" s="21"/>
-      <c r="L33" s="19"/>
-      <c r="M33" s="20"/>
-      <c r="N33" s="21"/>
-      <c r="O33" s="19"/>
-      <c r="P33" s="20"/>
-      <c r="Q33" s="21"/>
-      <c r="R33" s="19"/>
-      <c r="S33" s="20"/>
-      <c r="T33" s="21"/>
-      <c r="U33" s="19"/>
-      <c r="V33" s="20"/>
-      <c r="W33" s="20"/>
-      <c r="X33" s="21"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="16"/>
+      <c r="H33" s="17"/>
+      <c r="I33" s="18"/>
+      <c r="J33" s="19"/>
+      <c r="K33" s="20"/>
+      <c r="L33" s="18"/>
+      <c r="M33" s="19"/>
+      <c r="N33" s="20"/>
+      <c r="O33" s="18"/>
+      <c r="P33" s="19"/>
+      <c r="Q33" s="20"/>
+      <c r="R33" s="18"/>
+      <c r="S33" s="19"/>
+      <c r="T33" s="20"/>
+      <c r="U33" s="18"/>
+      <c r="V33" s="19"/>
+      <c r="W33" s="19"/>
+      <c r="X33" s="20"/>
       <c r="Y33" s="7"/>
       <c r="Z33" s="7"/>
     </row>
     <row r="34" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="8"/>
       <c r="B34" s="9"/>
-      <c r="C34" s="16"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="17"/>
-      <c r="H34" s="18"/>
-      <c r="I34" s="19"/>
-      <c r="J34" s="20"/>
-      <c r="K34" s="21"/>
-      <c r="L34" s="19"/>
-      <c r="M34" s="20"/>
-      <c r="N34" s="21"/>
-      <c r="O34" s="19"/>
-      <c r="P34" s="20"/>
-      <c r="Q34" s="21"/>
-      <c r="R34" s="19"/>
-      <c r="S34" s="20"/>
-      <c r="T34" s="21"/>
-      <c r="U34" s="19"/>
-      <c r="V34" s="20"/>
-      <c r="W34" s="20"/>
-      <c r="X34" s="21"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16"/>
+      <c r="G34" s="16"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="18"/>
+      <c r="J34" s="19"/>
+      <c r="K34" s="20"/>
+      <c r="L34" s="18"/>
+      <c r="M34" s="19"/>
+      <c r="N34" s="20"/>
+      <c r="O34" s="18"/>
+      <c r="P34" s="19"/>
+      <c r="Q34" s="20"/>
+      <c r="R34" s="18"/>
+      <c r="S34" s="19"/>
+      <c r="T34" s="20"/>
+      <c r="U34" s="18"/>
+      <c r="V34" s="19"/>
+      <c r="W34" s="19"/>
+      <c r="X34" s="20"/>
       <c r="Y34" s="7"/>
       <c r="Z34" s="7"/>
     </row>
     <row r="35" spans="1:26" ht="39.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="8"/>
       <c r="B35" s="9"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="23"/>
-      <c r="E35" s="23"/>
-      <c r="F35" s="23"/>
-      <c r="G35" s="23"/>
-      <c r="H35" s="24"/>
-      <c r="I35" s="25"/>
-      <c r="J35" s="26"/>
-      <c r="K35" s="27"/>
-      <c r="L35" s="25"/>
-      <c r="M35" s="26"/>
-      <c r="N35" s="27"/>
-      <c r="O35" s="25"/>
-      <c r="P35" s="26"/>
-      <c r="Q35" s="27"/>
-      <c r="R35" s="25"/>
-      <c r="S35" s="26"/>
-      <c r="T35" s="27"/>
-      <c r="U35" s="25"/>
-      <c r="V35" s="26"/>
-      <c r="W35" s="26"/>
-      <c r="X35" s="27"/>
+      <c r="C35" s="21"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="22"/>
+      <c r="H35" s="23"/>
+      <c r="I35" s="24"/>
+      <c r="J35" s="25"/>
+      <c r="K35" s="26"/>
+      <c r="L35" s="24"/>
+      <c r="M35" s="25"/>
+      <c r="N35" s="26"/>
+      <c r="O35" s="24"/>
+      <c r="P35" s="25"/>
+      <c r="Q35" s="26"/>
+      <c r="R35" s="24"/>
+      <c r="S35" s="25"/>
+      <c r="T35" s="26"/>
+      <c r="U35" s="24"/>
+      <c r="V35" s="25"/>
+      <c r="W35" s="25"/>
+      <c r="X35" s="26"/>
       <c r="Y35" s="7"/>
       <c r="Z35" s="7"/>
     </row>
     <row r="36" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="28"/>
-      <c r="B36" s="29"/>
-      <c r="C36" s="30"/>
-      <c r="D36" s="30"/>
-      <c r="E36" s="30"/>
-      <c r="F36" s="30"/>
-      <c r="G36" s="30"/>
-      <c r="H36" s="30"/>
+      <c r="A36" s="27"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="29"/>
+      <c r="H36" s="29"/>
       <c r="I36" s="7"/>
       <c r="J36" s="7"/>
       <c r="K36" s="7"/>

</xml_diff>